<commit_message>
atualizei os dados do 2Q26 da TLN
</commit_message>
<xml_diff>
--- a/analise_eua/energia_eletrica/talen/tln_indicators.xlsx
+++ b/analise_eua/energia_eletrica/talen/tln_indicators.xlsx
@@ -861,7 +861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1018,96 +1018,191 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46112</v>
+        <v>46203</v>
       </c>
       <c r="B2" t="n">
-        <v>231.11</v>
+        <v>-191.71</v>
       </c>
       <c r="C2" t="n">
-        <v>70.16</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="D2" t="n">
         <v>1.43</v>
       </c>
       <c r="E2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-12.32</v>
+      </c>
+      <c r="G2" t="n">
+        <v>10.91</v>
+      </c>
+      <c r="H2" t="n">
+        <v>17637534.44824219</v>
+      </c>
+      <c r="I2" t="n">
+        <v>9572</v>
+      </c>
+      <c r="J2" t="n">
+        <v>238</v>
+      </c>
+      <c r="K2" t="n">
+        <v>9334</v>
+      </c>
+      <c r="L2" t="n">
+        <v>12.27</v>
+      </c>
+      <c r="M2" t="n">
+        <v>5.78</v>
+      </c>
+      <c r="N2" t="n">
+        <v>35.44</v>
+      </c>
+      <c r="O2" t="n">
+        <v>15.47</v>
+      </c>
+      <c r="P2" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>-434</v>
+      </c>
+      <c r="R2" t="n">
+        <v>-2752</v>
+      </c>
+      <c r="S2" t="n">
+        <v>2397</v>
+      </c>
+      <c r="T2" t="n">
+        <v>-612</v>
+      </c>
+      <c r="U2" t="n">
+        <v>178</v>
+      </c>
+      <c r="V2" t="n">
+        <v>55</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" t="n">
+        <v>55</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>-288</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>34.56</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>24</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>270</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B3" t="n">
+        <v>231.11</v>
+      </c>
+      <c r="C3" t="n">
+        <v>70.16</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="E3" t="n">
         <v>276</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F3" t="n">
         <v>5.58</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G3" t="n">
         <v>13.57</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H3" t="n">
         <v>14560080.80108643</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I3" t="n">
         <v>6807</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J3" t="n">
         <v>1027</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K3" t="n">
         <v>5780</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L3" t="n">
         <v>8.18</v>
       </c>
-      <c r="M2" t="n">
+      <c r="M3" t="n">
         <v>5.39</v>
       </c>
-      <c r="N2" t="n">
+      <c r="N3" t="n">
         <v>28.77</v>
       </c>
-      <c r="O2" t="n">
+      <c r="O3" t="n">
         <v>19.29</v>
       </c>
-      <c r="P2" t="n">
+      <c r="P3" t="n">
         <v>6.61</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="Q3" t="n">
         <v>461</v>
       </c>
-      <c r="R2" t="n">
+      <c r="R3" t="n">
         <v>-72</v>
       </c>
-      <c r="S2" t="n">
+      <c r="S3" t="n">
         <v>-114</v>
       </c>
-      <c r="T2" t="n">
+      <c r="T3" t="n">
         <v>392</v>
       </c>
-      <c r="U2" t="n">
+      <c r="U3" t="n">
         <v>69</v>
       </c>
-      <c r="V2" t="n">
+      <c r="V3" t="n">
         <v>-39</v>
       </c>
-      <c r="W2" t="n">
-        <v>0</v>
-      </c>
-      <c r="X2" t="n">
+      <c r="W3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" t="n">
         <v>-39</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="Y3" t="n">
         <v>299</v>
       </c>
-      <c r="Z2" t="n">
+      <c r="Z3" t="n">
         <v>-30.13</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="AA3" t="n">
         <v>312</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="AB3" t="n">
         <v>590</v>
       </c>
-      <c r="AC2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE2" t="n">
+      <c r="AC3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>